<commit_message>
Master copy: point app at sri465inno/Agentic-QE-MVP, regenerate fixtures and demo artifacts, update README for hotel flows
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/08-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/08-report/CYC-3-cycle-report.xlsx
@@ -116,7 +116,7 @@
     <t>Narrative</t>
   </si>
   <si>
-    <t>Hotel booking baseline · End-to-end (baseline) worked from Jira initiative AQPI-1 (Jira export on GitHub), Jira epic AQPI-2, AQPI-6, AQPI-10, AQPI-14, AQPI-18, AQPI-23, AQPI-27 (Jira export on GitHub), Codebase sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) (pulled live from GitHub). The reviewed requirement set holds 128 requirements. 8 test cases are designed, 8 of them automated in 7 Playwright scripts. Execution ran 8 automated cases for real: 8 passed and 0 failed (pass rate 100%). No defects were raised.</t>
+    <t>Hotel booking baseline · End-to-end (baseline) worked from Jira initiative AQPI-1 (Jira export on GitHub), Jira epic AQPI-2, AQPI-6, AQPI-10, AQPI-14, AQPI-18, AQPI-23, AQPI-27 (Jira export on GitHub), Codebase sri465inno/Agentic-QE-MVP@demo/hotel-booking-platform (452df41) (pulled live from GitHub). The reviewed requirement set holds 128 requirements. 8 test cases are designed, 8 of them automated in 7 Playwright scripts. Execution ran 8 automated cases for real: 8 passed and 0 failed (pass rate 100%). No defects were raised.</t>
   </si>
   <si>
     <t>Narrative drafted by</t>
@@ -149,7 +149,7 @@
     <t>jira-export</t>
   </si>
   <si>
-    <t>Jira export on GitHub (sri465inno/uc-agentic-quality-engineering@demo/jira-export): Jira REST API v3 JSON of AQPI-1, exported from https://tcs-team-ou6drgfr.atlassian.net; no live Jira call was made</t>
+    <t>Jira export on GitHub (sri465inno/Agentic-QE-MVP@demo/jira-export): Jira REST API v3 JSON of AQPI-1, exported from https://tcs-team-ou6drgfr.atlassian.net; no live Jira call was made</t>
   </si>
   <si>
     <t>Jira epic</t>
@@ -158,19 +158,19 @@
     <t>AQPI-2, AQPI-6, AQPI-10, AQPI-14, AQPI-18, AQPI-23, AQPI-27</t>
   </si>
   <si>
-    <t>Jira export on GitHub (sri465inno/uc-agentic-quality-engineering@demo/jira-export): Jira REST API v3 JSON of AQPI-2, exported from https://tcs-team-ou6drgfr.atlassian.net; no live Jira call was made</t>
+    <t>Jira export on GitHub (sri465inno/Agentic-QE-MVP@demo/jira-export): Jira REST API v3 JSON of AQPI-2, exported from https://tcs-team-ou6drgfr.atlassian.net; no live Jira call was made</t>
   </si>
   <si>
     <t>Codebase</t>
   </si>
   <si>
-    <t>sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41)</t>
+    <t>sri465inno/Agentic-QE-MVP@demo/hotel-booking-platform (452df41)</t>
   </si>
   <si>
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) at 2026-10-05T16:27:05.604Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/Agentic-QE-MVP@demo/hotel-booking-platform (452df41) at 2026-10-05T16:43:53.537Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -2478,7 +2478,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-05T16:27:06.487Z</t>
+    <t>2026-10-05T16:43:54.326Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -10635,7 +10635,7 @@
         <v>679</v>
       </c>
       <c r="E2" s="2">
-        <v>1149</v>
+        <v>1074</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -10653,7 +10653,7 @@
         <v>679</v>
       </c>
       <c r="E3" s="2">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -10671,7 +10671,7 @@
         <v>679</v>
       </c>
       <c r="E4" s="2">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -10689,7 +10689,7 @@
         <v>679</v>
       </c>
       <c r="E5" s="2">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -10707,7 +10707,7 @@
         <v>679</v>
       </c>
       <c r="E6" s="2">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -10725,7 +10725,7 @@
         <v>679</v>
       </c>
       <c r="E7" s="2">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -10743,7 +10743,7 @@
         <v>679</v>
       </c>
       <c r="E8" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -10761,7 +10761,7 @@
         <v>679</v>
       </c>
       <c r="E9" s="2">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F9" s="2"/>
     </row>

</xml_diff>